<commit_message>
fix: graphic design labs require i3 8th gen+
</commit_message>
<xml_diff>
--- a/lab-standards/BWCCI-lab-standard.xlsx
+++ b/lab-standards/BWCCI-lab-standard.xlsx
@@ -2529,7 +2529,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2551,6 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -2595,8 +2593,6 @@
       <c r="F8" s="11" t="n"/>
       <c r="G8" s="12" t="n"/>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -2604,7 +2600,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="115.65" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -2616,7 +2611,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="26.85" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
@@ -2952,6 +2946,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2974,6 +2969,7 @@
         <v>25</v>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -3016,6 +3012,8 @@
       <c r="F8" s="11" t="n"/>
       <c r="G8" s="12" t="n"/>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -3023,6 +3021,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="115.65" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -3034,6 +3033,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="26.85" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Laptop/ Desktop (Minimum Intel core i5 or Intel core i3 6 gen/above, or AMD Ryzen 5/ similar spec; Ram: minimum 8 - 16 GB; Display: FHD monitor; Graphic Card: dedicated GPU 2GB; High Speed Internet (Minimum 10 Mbps); Graphic Design Software 
+          <t>Laptop/ Desktop (Minimum Intel core i5 or Intel core i3 8 gen/above, or AMD Ryzen 5/ similar spec; Ram: minimum 8 - 16 GB; Display: FHD monitor; Graphic Card: dedicated GPU 2GB; High Speed Internet (Minimum 10 Mbps); Graphic Design Software 
 (Photoshop CC, Illustrator CC, InDesign, After Effects, CorelDraw); 3D Design Software (Blender, Cinema 4D or Autodesk Maya)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
fix: AMD Ryzen similar spec in design/DM labs
</commit_message>
<xml_diff>
--- a/lab-standards/BWCCI-lab-standard.xlsx
+++ b/lab-standards/BWCCI-lab-standard.xlsx
@@ -2529,6 +2529,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2551,6 +2552,7 @@
         <v>25</v>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -2593,6 +2595,8 @@
       <c r="F8" s="11" t="n"/>
       <c r="G8" s="12" t="n"/>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -2600,6 +2604,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="115.65" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -2611,6 +2616,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="26.85" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
@@ -2727,7 +2733,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Computers/Laptop: (Minimum Intel core i5 or Intel core i3 6 gen/above, or AMD similar spec, 8GB RAM (16GB preferred), 500GB SSD storage (1TB preferred), High-resolution monitors (19/20-inch minimum, with color accuracy).</t>
+          <t>Computers/Laptop: (Minimum Intel core i5 or Intel core i3 6 gen/above, or AMD Ryzen similar spec, 8GB RAM (16GB preferred), 500GB SSD storage (1TB preferred), High-resolution monitors (19/20-inch minimum, with color accuracy).</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
@@ -3078,7 +3084,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Laptop/ Desktop (Minimum Intel core i5 or Intel core i3 8 gen/above, or AMD Ryzen 5/ similar spec; Ram: minimum 8 - 16 GB; Display: FHD monitor; Graphic Card: dedicated GPU 2GB; High Speed Internet (Minimum 10 Mbps); Graphic Design Software 
+          <t>Laptop/ Desktop (Minimum Intel core i5 or Intel core i3 8 gen/above, or AMD Ryzen similar spec; Ram: minimum 8 - 16 GB; Display: FHD monitor; Graphic Card: dedicated GPU 2GB; High Speed Internet (Minimum 10 Mbps); Graphic Design Software 
 (Photoshop CC, Illustrator CC, InDesign, After Effects, CorelDraw); 3D Design Software (Blender, Cinema 4D or Autodesk Maya)</t>
         </is>
       </c>

</xml_diff>